<commit_message>
Coleta automática em 10-01-2026 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-01-2026 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 12-01-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 13-01-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 15-01-2026 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 16-01-2026 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-01-2026 20:23
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,82 +417,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>marca</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>produto</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>preco</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>data_coleta</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>preco_antigo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>desconto</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>disponibilidade</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>produto_id</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>sku_id</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>metodo</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>medicamento_base</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>variacao</t>
         </is>

</xml_diff>

<commit_message>
Coleta automática em 22-01-2026 20:18
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-01-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-01-2026 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-01-2026 20:29
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-01-2026 20:20
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-01-2026 20:22
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-01-2026 20:20
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-02-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 04-02-2026 20:25
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 06-02-2026 20:24
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-02-2026 20:18
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-02-2026 20:34
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-02-2026 20:31
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 12-02-2026 20:26
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 15-02-2026 20:18
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 16-02-2026 20:21
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-02-2026 20:28
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-02-2026 20:31
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-02-2026 20:22
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-02-2026 20:37
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-02-2026 20:26
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-02-2026 20:27
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 06-03-2026 20:24
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-03-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 10-03-2026 20:26
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-03-2026 20:27
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 12-03-2026 20:27
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 16-03-2026 20:31
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-03-2026 20:28
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-03-2026 20:30
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-03-2026 20:18
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-03-2026 20:31
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-03-2026 20:23
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 31-03-2026 20:36
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-04-2026 20:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 04-04-2026 20:22
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-04-2026 20:39
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-04-2026 20:36
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-04-2026 20:44
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 10-04-2026 20:29
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-04-2026 20:24
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 13-04-2026 20:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 14-04-2026 20:46
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 15-04-2026 20:41
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 16-04-2026 20:45
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-04-2026 20:39
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-04-2026 20:43
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-04-2026 20:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-04-2026 20:31
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-04-2026 20:53
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 28-04-2026 21:03
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 02-05-2026 20:34
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 03-05-2026 20:35
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 04-05-2026 21:01
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 05-05-2026 20:55
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 06-05-2026 21:05
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-05-2026 20:37
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 10-05-2026 20:40
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-05-2026 21:13
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 13-05-2026 21:19
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 14-05-2026 21:06
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 15-05-2026 20:52
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-05-2026 20:43
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-05-2026 21:05
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-05-2026 21:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-05-2026 21:33
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-05-2026 21:30
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-05-2026 21:36
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-05-2026 20:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-06-2026 22:33
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 04-06-2026 21:26
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 05-06-2026 21:19
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 06-06-2026 20:57
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-06-2026 21:59
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 14-06-2026 21:02
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 16-06-2026 22:10
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-06-2026 21:56
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-06-2026 21:08
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-06-2026 21:27
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-06-2026 21:21
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 28-06-2026 20:55
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-06-2026 21:20
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-06-2026 21:27
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 02-07-2026 20:54
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 03-07-2026 20:56
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-07-2026 21:20
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-07-2026 20:41
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 14-07-2026 20:53
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 15-07-2026 20:53
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 16-07-2026 20:48
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-07-2026 20:46
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-07-2026 20:40
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-07-2026 20:41
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-07-2026 21:01
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-07-2026 20:56
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-07-2026 20:55
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-07-2026 20:59
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-07-2026 20:44
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 28-07-2026 21:02
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-07-2026 20:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 31-07-2026 20:56
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-08-2026 20:45
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 02-08-2026 20:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-08-2026 00:56
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-08-2026 20:32
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-08-2026 20:19
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-08-2026 20:37
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 12-08-2026 20:35
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 14-08-2026 20:25
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 15-08-2026 20:14
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 16-08-2026 20:14
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-08-2026 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-08-2026 20:21
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-08-2026 20:18
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-08-2026 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-08-2026 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-08-2026 20:20
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-08-2026 22:40
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 28-08-2026 03:59
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-08-2026 02:37
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-08-2026 22:10
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-08-2026 22:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-09-2026 22:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 03-09-2026 22:03
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 05-09-2026 21:52
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>topspot</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 06-09-2026 21:53
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_cobasi_20250926_182214.xlsx
@@ -5070,7 +5070,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5140,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>topspot</t>
         </is>
       </c>
     </row>

</xml_diff>